<commit_message>
#160 Supplier BOM Edit
</commit_message>
<xml_diff>
--- a/Deliverables/SM_Top Board/_BOM/Supplier BOM-TOP Board.xlsx
+++ b/Deliverables/SM_Top Board/_BOM/Supplier BOM-TOP Board.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25928"/>
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eSpark-Consultants\ColeBenson-SmartMotors\Deliverables\SM_Top Board\_BOM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB218B4B-544C-4669-9561-650772D5196D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -74,9 +73,6 @@
     <t>C36</t>
   </si>
   <si>
-    <t>C37</t>
-  </si>
-  <si>
     <t>C42</t>
   </si>
   <si>
@@ -152,9 +148,6 @@
     <t>R6, R7, R8, R9</t>
   </si>
   <si>
-    <t>R10, R11, R12, R13</t>
-  </si>
-  <si>
     <t>R21</t>
   </si>
   <si>
@@ -359,9 +352,6 @@
     <t>RES SMD 47OHM 0.1W 0603</t>
   </si>
   <si>
-    <t>0.033Ω ±1% 2W ±1800ppm/°C 2512 Low Resistors &amp; Current Sense Resistors - Surface Mount RoHS</t>
-  </si>
-  <si>
     <t>RES SMD 150OHM 1/10W 0603</t>
   </si>
   <si>
@@ -854,9 +844,6 @@
     <t>47R</t>
   </si>
   <si>
-    <t>33m</t>
-  </si>
-  <si>
     <t>150R</t>
   </si>
   <si>
@@ -1034,9 +1021,6 @@
     <t>AO4882-MS</t>
   </si>
   <si>
-    <t>LR2512-22R033F4</t>
-  </si>
-  <si>
     <t>ARG03FTC1273</t>
   </si>
   <si>
@@ -1098,9 +1082,6 @@
   </si>
   <si>
     <t>RES SMD 22HM 1/10W 0603</t>
-  </si>
-  <si>
-    <t>C5, C6, C14, C23, C24, C29, C34, C35</t>
   </si>
   <si>
     <t>C43</t>
@@ -1371,11 +1352,29 @@
   <si>
     <t>Ali-E</t>
   </si>
+  <si>
+    <t>C5, C6, C14, C29, C34, C35</t>
+  </si>
+  <si>
+    <t>C23, C24, C37</t>
+  </si>
+  <si>
+    <t>R12, R13</t>
+  </si>
+  <si>
+    <t>2W 50mΩ ±1% 2512 Current Sense Resistors/Shunt Resistors ROHS</t>
+  </si>
+  <si>
+    <t>CRH2512FR050E04Z</t>
+  </si>
+  <si>
+    <t>50mR</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
   </numFmts>
@@ -2492,7 +2491,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:Q91"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2537,7 +2536,7 @@
       </c>
       <c r="E2" s="8"/>
       <c r="F2" s="42" t="s">
-        <v>317</v>
+        <v>313</v>
       </c>
       <c r="G2" s="9"/>
       <c r="H2" s="3"/>
@@ -2557,7 +2556,7 @@
       </c>
       <c r="E3" s="10"/>
       <c r="F3" s="43" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="G3" s="10"/>
       <c r="H3" s="4"/>
@@ -2577,7 +2576,7 @@
       </c>
       <c r="E4" s="10"/>
       <c r="F4" s="44" t="s">
-        <v>316</v>
+        <v>312</v>
       </c>
       <c r="G4" s="11"/>
       <c r="H4" s="6"/>
@@ -2660,40 +2659,40 @@
         <v>4</v>
       </c>
       <c r="C9" s="26" t="s">
-        <v>309</v>
+        <v>305</v>
       </c>
       <c r="D9" s="26" t="s">
         <v>5</v>
       </c>
       <c r="E9" s="27" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="F9" s="26" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="G9" s="27" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="H9" s="26" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="I9" s="27" t="s">
-        <v>393</v>
+        <v>387</v>
       </c>
       <c r="J9" s="26" t="s">
-        <v>291</v>
+        <v>287</v>
       </c>
       <c r="K9" s="28" t="s">
-        <v>318</v>
+        <v>314</v>
       </c>
       <c r="L9" s="28" t="s">
-        <v>394</v>
+        <v>388</v>
       </c>
       <c r="M9" s="28" t="s">
-        <v>395</v>
+        <v>389</v>
       </c>
       <c r="N9" s="28" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
     </row>
     <row r="10" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2703,31 +2702,31 @@
         <v>1</v>
       </c>
       <c r="C10" s="46" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="D10" s="29" t="s">
         <v>6</v>
       </c>
       <c r="E10" s="30" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="F10" s="29" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="G10" s="29" t="s">
-        <v>391</v>
+        <v>385</v>
       </c>
       <c r="H10" s="29" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="I10" s="30" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="J10" s="29">
         <v>1</v>
       </c>
       <c r="K10" s="50" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="L10" s="33">
         <v>1.2</v>
@@ -2736,7 +2735,7 @@
         <v>1.2</v>
       </c>
       <c r="N10" s="33" t="s">
-        <v>396</v>
+        <v>390</v>
       </c>
     </row>
     <row r="11" spans="1:14" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2746,31 +2745,31 @@
         <v>2</v>
       </c>
       <c r="C11" s="63" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="D11" s="64" t="s">
-        <v>377</v>
+        <v>371</v>
       </c>
       <c r="E11" s="65" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="F11" s="64" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="G11" s="65" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="H11" s="64" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="I11" s="65" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="J11" s="64">
         <v>15</v>
       </c>
       <c r="K11" s="67" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L11" s="66">
         <v>2.5000000000000001E-3</v>
@@ -2779,7 +2778,7 @@
         <v>0.25</v>
       </c>
       <c r="N11" s="66" t="s">
-        <v>376</v>
+        <v>370</v>
       </c>
     </row>
     <row r="12" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -2789,31 +2788,31 @@
         <v>3</v>
       </c>
       <c r="C12" s="48" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="D12" s="29" t="s">
-        <v>373</v>
+        <v>367</v>
       </c>
       <c r="E12" s="30" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="F12" s="29" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="G12" s="30" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="H12" s="29" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="I12" s="30" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="J12" s="68">
         <v>2</v>
       </c>
       <c r="K12" s="50" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L12" s="33">
         <v>1.2999999999999999E-3</v>
@@ -2830,31 +2829,31 @@
         <v>4</v>
       </c>
       <c r="C13" s="47" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="D13" s="31" t="s">
-        <v>347</v>
+        <v>342</v>
       </c>
       <c r="E13" s="32" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="F13" s="31" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="G13" s="32" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="H13" s="31" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="I13" s="32" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="J13" s="69">
         <v>1</v>
       </c>
       <c r="K13" s="51" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L13" s="34">
         <v>2.6499999999999999E-2</v>
@@ -2871,31 +2870,31 @@
         <v>5</v>
       </c>
       <c r="C14" s="48" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="D14" s="29" t="s">
-        <v>355</v>
+        <v>395</v>
       </c>
       <c r="E14" s="30" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="F14" s="29" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="G14" s="30" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="H14" s="29" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="I14" s="30" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="J14" s="29">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K14" s="50" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L14" s="33">
         <v>5.96E-2</v>
@@ -2912,31 +2911,31 @@
         <v>6</v>
       </c>
       <c r="C15" s="47" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="D15" s="31" t="s">
-        <v>372</v>
+        <v>366</v>
       </c>
       <c r="E15" s="32" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F15" s="31" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="G15" s="32" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="H15" s="31" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="I15" s="32" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="J15" s="69">
         <v>3</v>
       </c>
       <c r="K15" s="51" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L15" s="34">
         <v>4.8999999999999998E-3</v>
@@ -2953,31 +2952,31 @@
         <v>7</v>
       </c>
       <c r="C16" s="48" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="D16" s="29" t="s">
-        <v>371</v>
+        <v>365</v>
       </c>
       <c r="E16" s="30" t="s">
-        <v>370</v>
+        <v>364</v>
       </c>
       <c r="F16" s="29" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="G16" s="81" t="s">
-        <v>349</v>
+        <v>344</v>
       </c>
       <c r="H16" s="68" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="I16" s="30" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="J16" s="29">
         <v>6</v>
       </c>
       <c r="K16" s="50" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L16" s="33">
         <v>3.6900000000000002E-2</v>
@@ -2994,31 +2993,31 @@
         <v>8</v>
       </c>
       <c r="C17" s="47" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="D17" s="31" t="s">
         <v>7</v>
       </c>
       <c r="E17" s="32" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="F17" s="31" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="G17" s="32" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="H17" s="31" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="I17" s="32" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="J17" s="31">
         <v>1</v>
       </c>
       <c r="K17" s="51" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L17" s="34">
         <v>3.0999999999999999E-3</v>
@@ -3035,31 +3034,31 @@
         <v>9</v>
       </c>
       <c r="C18" s="82" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="D18" s="83" t="s">
-        <v>322</v>
+        <v>318</v>
       </c>
       <c r="E18" s="84" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F18" s="83" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="G18" s="83" t="s">
-        <v>320</v>
+        <v>316</v>
       </c>
       <c r="H18" s="83" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="I18" s="84" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="J18" s="83">
         <v>8</v>
       </c>
       <c r="K18" s="85" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L18" s="76">
         <v>2.3199999999999998E-2</v>
@@ -3076,31 +3075,31 @@
         <v>10</v>
       </c>
       <c r="C19" s="86" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="D19" s="87" t="s">
         <v>8</v>
       </c>
       <c r="E19" s="88" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="F19" s="87" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="G19" s="87" t="s">
-        <v>321</v>
+        <v>317</v>
       </c>
       <c r="H19" s="87" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="I19" s="88" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="J19" s="87">
         <v>1</v>
       </c>
       <c r="K19" s="90" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L19" s="89">
         <v>4.7000000000000002E-3</v>
@@ -3117,31 +3116,31 @@
         <v>11</v>
       </c>
       <c r="C20" s="82" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="D20" s="83" t="s">
         <v>9</v>
       </c>
       <c r="E20" s="84" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="F20" s="83" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="G20" s="83" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="H20" s="83" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="I20" s="84" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="J20" s="83">
         <v>1</v>
       </c>
       <c r="K20" s="85" t="s">
-        <v>397</v>
+        <v>391</v>
       </c>
       <c r="L20" s="76">
         <v>0.16109999999999999</v>
@@ -3158,31 +3157,31 @@
         <v>12</v>
       </c>
       <c r="C21" s="86" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="D21" s="87" t="s">
         <v>10</v>
       </c>
       <c r="E21" s="88" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="F21" s="87" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="G21" s="88" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="H21" s="87" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="I21" s="88" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="J21" s="87">
         <v>2</v>
       </c>
       <c r="K21" s="90" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L21" s="89">
         <v>6.4999999999999997E-3</v>
@@ -3199,31 +3198,31 @@
         <v>13</v>
       </c>
       <c r="C22" s="48" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="D22" s="29" t="s">
         <v>11</v>
       </c>
       <c r="E22" s="30" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F22" s="29" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="G22" s="30" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="H22" s="29" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="I22" s="30" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="J22" s="29">
         <v>1</v>
       </c>
       <c r="K22" s="50" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L22" s="33">
         <v>3.1099999999999999E-2</v>
@@ -3240,31 +3239,31 @@
         <v>14</v>
       </c>
       <c r="C23" s="47" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="D23" s="31" t="s">
-        <v>346</v>
+        <v>341</v>
       </c>
       <c r="E23" s="32" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F23" s="31" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="G23" s="32" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="H23" s="31" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="I23" s="32" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="J23" s="31">
         <v>1</v>
       </c>
       <c r="K23" s="51" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L23" s="34">
         <v>1.7399999999999999E-2</v>
@@ -3281,31 +3280,31 @@
         <v>15</v>
       </c>
       <c r="C24" s="48" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="D24" s="29" t="s">
         <v>12</v>
       </c>
       <c r="E24" s="30" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F24" s="29" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="G24" s="29" t="s">
-        <v>323</v>
+        <v>319</v>
       </c>
       <c r="H24" s="29" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="I24" s="30" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="J24" s="29">
         <v>1</v>
       </c>
       <c r="K24" s="50" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L24" s="33">
         <v>4.4000000000000003E-3</v>
@@ -3322,31 +3321,31 @@
         <v>16</v>
       </c>
       <c r="C25" s="47" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="D25" s="31" t="s">
-        <v>13</v>
+        <v>396</v>
       </c>
       <c r="E25" s="32" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="F25" s="31" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="G25" s="32" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="H25" s="31" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="I25" s="32" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="J25" s="31">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K25" s="51" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L25" s="34">
         <v>2.5000000000000001E-3</v>
@@ -3363,31 +3362,31 @@
         <v>17</v>
       </c>
       <c r="C26" s="82" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="D26" s="83" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E26" s="91" t="s">
-        <v>348</v>
+        <v>343</v>
       </c>
       <c r="F26" s="83" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="G26" s="91" t="s">
-        <v>369</v>
+        <v>363</v>
       </c>
       <c r="H26" s="92" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="I26" s="91" t="s">
-        <v>357</v>
+        <v>351</v>
       </c>
       <c r="J26" s="83">
         <v>1</v>
       </c>
       <c r="K26" s="85" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L26" s="76">
         <v>3.0000000000000001E-3</v>
@@ -3404,31 +3403,31 @@
         <v>18</v>
       </c>
       <c r="C27" s="86" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="D27" s="87" t="s">
-        <v>356</v>
+        <v>350</v>
       </c>
       <c r="E27" s="88" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="F27" s="87" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="G27" s="88" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="H27" s="87" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="I27" s="88" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="J27" s="87">
         <v>1</v>
       </c>
       <c r="K27" s="90" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L27" s="89">
         <v>0.30830000000000002</v>
@@ -3445,31 +3444,31 @@
         <v>19</v>
       </c>
       <c r="C28" s="48" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="D28" s="29" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E28" s="30" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="F28" s="29" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="G28" s="30" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="H28" s="29" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="I28" s="30" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="J28" s="29">
         <v>1</v>
       </c>
       <c r="K28" s="50" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L28" s="33">
         <v>1.365</v>
@@ -3486,31 +3485,31 @@
         <v>20</v>
       </c>
       <c r="C29" s="47" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="D29" s="31" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E29" s="32" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="F29" s="31" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="G29" s="31" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="H29" s="31" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="I29" s="32" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="J29" s="31">
         <v>1</v>
       </c>
       <c r="K29" s="51" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L29" s="34">
         <v>0.35959999999999998</v>
@@ -3527,31 +3526,31 @@
         <v>21</v>
       </c>
       <c r="C30" s="48" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="D30" s="29" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E30" s="30" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="F30" s="29" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="G30" s="30" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="H30" s="29" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="I30" s="30" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="J30" s="29">
         <v>1</v>
       </c>
       <c r="K30" s="50" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L30" s="33">
         <v>2.3999999999999998E-3</v>
@@ -3568,31 +3567,31 @@
         <v>22</v>
       </c>
       <c r="C31" s="86" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="D31" s="87" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E31" s="88" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="F31" s="87" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="G31" s="88" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="H31" s="87" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="I31" s="88" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="J31" s="87">
         <v>4</v>
       </c>
       <c r="K31" s="90" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L31" s="89">
         <v>5.1000000000000004E-3</v>
@@ -3609,31 +3608,31 @@
         <v>23</v>
       </c>
       <c r="C32" s="82" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="D32" s="83" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E32" s="84" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="F32" s="83" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="G32" s="84" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="H32" s="83" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="I32" s="84" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="J32" s="83">
         <v>1</v>
       </c>
       <c r="K32" s="85" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L32" s="76">
         <v>3.9300000000000002E-2</v>
@@ -3650,31 +3649,31 @@
         <v>24</v>
       </c>
       <c r="C33" s="86" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="D33" s="87" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E33" s="88" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="F33" s="87" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="G33" s="88" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="H33" s="87" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="I33" s="88" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="J33" s="87">
         <v>1</v>
       </c>
       <c r="K33" s="90" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L33" s="89">
         <v>7.1900000000000006E-2</v>
@@ -3691,31 +3690,31 @@
         <v>25</v>
       </c>
       <c r="C34" s="82" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="D34" s="83" t="s">
-        <v>374</v>
+        <v>368</v>
       </c>
       <c r="E34" s="84" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="F34" s="83" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="G34" s="84" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="H34" s="83" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="I34" s="84" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="J34" s="83">
         <v>2</v>
       </c>
       <c r="K34" s="85" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L34" s="76">
         <v>2.63E-2</v>
@@ -3732,31 +3731,31 @@
         <v>26</v>
       </c>
       <c r="C35" s="70" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="D35" s="71" t="s">
-        <v>358</v>
+        <v>352</v>
       </c>
       <c r="E35" s="72" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="F35" s="71" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="G35" s="71" t="s">
-        <v>324</v>
+        <v>320</v>
       </c>
       <c r="H35" s="71" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="I35" s="72" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="J35" s="73">
         <v>8</v>
       </c>
       <c r="K35" s="75" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="L35" s="74">
         <v>0.42</v>
@@ -3765,7 +3764,7 @@
         <v>3.36</v>
       </c>
       <c r="N35" s="66" t="s">
-        <v>359</v>
+        <v>353</v>
       </c>
       <c r="Q35" s="95"/>
     </row>
@@ -3776,31 +3775,31 @@
         <v>27</v>
       </c>
       <c r="C36" s="82" t="s">
-        <v>303</v>
+        <v>299</v>
       </c>
       <c r="D36" s="83" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E36" s="84" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="F36" s="83" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="G36" s="83" t="s">
-        <v>325</v>
+        <v>321</v>
       </c>
       <c r="H36" s="83" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="I36" s="84" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="J36" s="83">
         <v>1</v>
       </c>
       <c r="K36" s="85" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L36" s="76">
         <v>6.7699999999999996E-2</v>
@@ -3817,31 +3816,31 @@
         <v>28</v>
       </c>
       <c r="C37" s="86" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
       <c r="D37" s="87" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E37" s="88" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="F37" s="87" t="s">
-        <v>293</v>
+        <v>289</v>
       </c>
       <c r="G37" s="88" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="H37" s="87" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="I37" s="88" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="J37" s="87">
         <v>4</v>
       </c>
       <c r="K37" s="90" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L37" s="89">
         <v>2.8000000000000001E-2</v>
@@ -3858,31 +3857,31 @@
         <v>29</v>
       </c>
       <c r="C38" s="82" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="D38" s="83" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E38" s="84" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="F38" s="83" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="G38" s="83" t="s">
-        <v>326</v>
+        <v>322</v>
       </c>
       <c r="H38" s="83" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="I38" s="84" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="J38" s="83">
         <v>1</v>
       </c>
       <c r="K38" s="85" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L38" s="76">
         <v>0.60140000000000005</v>
@@ -3899,31 +3898,31 @@
         <v>30</v>
       </c>
       <c r="C39" s="86" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="D39" s="87" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E39" s="88" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="F39" s="87" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="G39" s="87" t="s">
-        <v>327</v>
+        <v>323</v>
       </c>
       <c r="H39" s="87" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="I39" s="88" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="J39" s="87">
         <v>2</v>
       </c>
       <c r="K39" s="90" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L39" s="89">
         <v>0.75729999999999997</v>
@@ -3940,31 +3939,31 @@
         <v>31</v>
       </c>
       <c r="C40" s="82" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="D40" s="83" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E40" s="84" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="F40" s="83" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="G40" s="84" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="H40" s="83" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="I40" s="84" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="J40" s="83">
         <v>1</v>
       </c>
       <c r="K40" s="85" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="L40" s="76">
         <v>1.8</v>
@@ -3981,31 +3980,31 @@
         <v>32</v>
       </c>
       <c r="C41" s="86" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="D41" s="87" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E41" s="88" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="F41" s="87" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="G41" s="88" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="H41" s="87" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="I41" s="88" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="J41" s="87">
         <v>1</v>
       </c>
       <c r="K41" s="90" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L41" s="89">
         <v>5.1200000000000002E-2</v>
@@ -4022,31 +4021,31 @@
         <v>33</v>
       </c>
       <c r="C42" s="86" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="D42" s="87" t="s">
-        <v>387</v>
+        <v>381</v>
       </c>
       <c r="E42" s="88" t="s">
-        <v>389</v>
+        <v>383</v>
       </c>
       <c r="F42" s="87" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="G42" s="88" t="s">
-        <v>388</v>
+        <v>382</v>
       </c>
       <c r="H42" s="87" t="s">
-        <v>390</v>
+        <v>384</v>
       </c>
       <c r="I42" s="88" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="J42" s="87">
         <v>1</v>
       </c>
       <c r="K42" s="90" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L42" s="89">
         <v>0.21920000000000001</v>
@@ -4063,31 +4062,31 @@
         <v>34</v>
       </c>
       <c r="C43" s="82" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
       <c r="D43" s="83" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E43" s="84" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F43" s="83" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="G43" s="84" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="H43" s="83" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="I43" s="84" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="J43" s="83">
         <v>1</v>
       </c>
       <c r="K43" s="85" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L43" s="76">
         <v>0.47249999999999998</v>
@@ -4104,31 +4103,31 @@
         <v>35</v>
       </c>
       <c r="C44" s="86" t="s">
-        <v>302</v>
+        <v>298</v>
       </c>
       <c r="D44" s="87" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E44" s="88" t="s">
-        <v>362</v>
+        <v>356</v>
       </c>
       <c r="F44" s="87" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="G44" s="88" t="s">
-        <v>361</v>
+        <v>355</v>
       </c>
       <c r="H44" s="87" t="s">
-        <v>351</v>
+        <v>346</v>
       </c>
       <c r="I44" s="88" t="s">
-        <v>360</v>
+        <v>354</v>
       </c>
       <c r="J44" s="87">
         <v>1</v>
       </c>
       <c r="K44" s="90" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L44" s="89">
         <v>9.7500000000000003E-2</v>
@@ -4145,31 +4144,31 @@
         <v>36</v>
       </c>
       <c r="C45" s="82" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="D45" s="83" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E45" s="84" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F45" s="83" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="G45" s="84" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="H45" s="83" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="I45" s="84" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="J45" s="83">
         <v>1</v>
       </c>
       <c r="K45" s="85" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="L45" s="76">
         <v>0.7</v>
@@ -4186,31 +4185,31 @@
         <v>37</v>
       </c>
       <c r="C46" s="86" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="D46" s="87" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E46" s="88" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F46" s="87" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="G46" s="88" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="H46" s="87" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="I46" s="88" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="J46" s="87">
         <v>1</v>
       </c>
       <c r="K46" s="90" t="s">
-        <v>330</v>
+        <v>326</v>
       </c>
       <c r="L46" s="89">
         <v>0.08</v>
@@ -4227,31 +4226,31 @@
         <v>38</v>
       </c>
       <c r="C47" s="86" t="s">
-        <v>378</v>
+        <v>372</v>
       </c>
       <c r="D47" s="87" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="E47" s="88" t="s">
-        <v>380</v>
+        <v>374</v>
       </c>
       <c r="F47" s="87" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="G47" s="88" t="s">
-        <v>381</v>
+        <v>375</v>
       </c>
       <c r="H47" s="87" t="s">
-        <v>382</v>
+        <v>376</v>
       </c>
       <c r="I47" s="88" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="J47" s="87">
         <v>1</v>
       </c>
       <c r="K47" s="90" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="L47" s="89">
         <v>0.66</v>
@@ -4260,7 +4259,7 @@
         <v>0.66</v>
       </c>
       <c r="N47" s="61" t="s">
-        <v>379</v>
+        <v>373</v>
       </c>
     </row>
     <row r="48" spans="1:17" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -4270,31 +4269,31 @@
         <v>39</v>
       </c>
       <c r="C48" s="82" t="s">
-        <v>304</v>
+        <v>300</v>
       </c>
       <c r="D48" s="83" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E48" s="84" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="F48" s="83" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="G48" s="84" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="H48" s="83" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="I48" s="84" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="J48" s="83">
         <v>2</v>
       </c>
       <c r="K48" s="85" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="L48" s="76">
         <v>1.5</v>
@@ -4311,25 +4310,25 @@
         <v>40</v>
       </c>
       <c r="C49" s="77" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="D49" s="78" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E49" s="79" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="F49" s="78" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="G49" s="79" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="H49" s="78" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="I49" s="79" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="J49" s="78">
         <v>4</v>
@@ -4337,10 +4336,10 @@
       <c r="K49" s="52"/>
       <c r="L49" s="52"/>
       <c r="M49" s="52" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="N49" s="52" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
     </row>
     <row r="50" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -4350,31 +4349,31 @@
         <v>41</v>
       </c>
       <c r="C50" s="82" t="s">
-        <v>305</v>
+        <v>301</v>
       </c>
       <c r="D50" s="83" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E50" s="84" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="F50" s="83" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="G50" s="83" t="s">
-        <v>399</v>
+        <v>393</v>
       </c>
       <c r="H50" s="83" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="I50" s="84" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="J50" s="83">
         <v>4</v>
       </c>
       <c r="K50" s="85" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L50" s="76">
         <v>1.47E-2</v>
@@ -4391,31 +4390,31 @@
         <v>42</v>
       </c>
       <c r="C51" s="86" t="s">
-        <v>307</v>
+        <v>303</v>
       </c>
       <c r="D51" s="87" t="s">
-        <v>353</v>
+        <v>348</v>
       </c>
       <c r="E51" s="88" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="F51" s="87" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="G51" s="87" t="s">
-        <v>332</v>
+        <v>328</v>
       </c>
       <c r="H51" s="87" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="I51" s="88" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="J51" s="87">
         <v>4</v>
       </c>
       <c r="K51" s="90" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L51" s="89">
         <v>0.39140000000000003</v>
@@ -4432,31 +4431,31 @@
         <v>43</v>
       </c>
       <c r="C52" s="82" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="D52" s="83" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E52" s="84" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="F52" s="83" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="G52" s="84" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="H52" s="83" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="I52" s="84" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="J52" s="83">
         <v>2</v>
       </c>
       <c r="K52" s="85" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L52" s="76">
         <v>1E-3</v>
@@ -4473,31 +4472,31 @@
         <v>44</v>
       </c>
       <c r="C53" s="86" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="D53" s="87" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E53" s="88" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="F53" s="87" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="G53" s="88" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="H53" s="87" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="I53" s="88" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="J53" s="87">
         <v>1</v>
       </c>
       <c r="K53" s="90" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L53" s="89">
         <v>1.2999999999999999E-3</v>
@@ -4514,31 +4513,31 @@
         <v>45</v>
       </c>
       <c r="C54" s="82" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="D54" s="83" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="E54" s="84" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F54" s="83" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="G54" s="84" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="H54" s="83" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="I54" s="84" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="J54" s="83">
         <v>1</v>
       </c>
       <c r="K54" s="85" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L54" s="76">
         <v>8.0000000000000004E-4</v>
@@ -4555,31 +4554,31 @@
         <v>46</v>
       </c>
       <c r="C55" s="86" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="D55" s="87" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E55" s="88" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="F55" s="87" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="G55" s="88" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="H55" s="87" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="I55" s="88" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="J55" s="87">
         <v>2</v>
       </c>
       <c r="K55" s="90" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L55" s="89">
         <v>1.1999999999999999E-3</v>
@@ -4596,31 +4595,31 @@
         <v>47</v>
       </c>
       <c r="C56" s="82" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="D56" s="83" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="E56" s="84" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="F56" s="83" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="G56" s="84" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="H56" s="83" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="I56" s="84" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="J56" s="83">
         <v>4</v>
       </c>
       <c r="K56" s="85" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L56" s="76">
         <v>1.1999999999999999E-3</v>
@@ -4630,41 +4629,41 @@
       </c>
       <c r="N56" s="76"/>
     </row>
-    <row r="57" spans="1:14" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:14" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="1"/>
       <c r="B57" s="41">
         <f t="shared" si="0"/>
         <v>48</v>
       </c>
       <c r="C57" s="86" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="D57" s="87" t="s">
-        <v>39</v>
-      </c>
-      <c r="E57" s="88" t="s">
-        <v>108</v>
+        <v>397</v>
+      </c>
+      <c r="E57" s="31" t="s">
+        <v>398</v>
       </c>
       <c r="F57" s="87" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="G57" s="87" t="s">
-        <v>333</v>
+        <v>399</v>
       </c>
       <c r="H57" s="87" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="I57" s="88" t="s">
-        <v>273</v>
+        <v>400</v>
       </c>
       <c r="J57" s="87">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K57" s="90" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L57" s="89">
-        <v>8.8300000000000003E-2</v>
+        <v>2.9100000000000001E-2</v>
       </c>
       <c r="M57" s="89">
         <v>0.4415</v>
@@ -4678,31 +4677,31 @@
         <v>49</v>
       </c>
       <c r="C58" s="48" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="D58" s="29" t="s">
-        <v>342</v>
+        <v>337</v>
       </c>
       <c r="E58" s="29" t="s">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="F58" s="29" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="G58" s="29" t="s">
-        <v>344</v>
+        <v>339</v>
       </c>
       <c r="H58" s="29" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="I58" s="29" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="J58" s="29">
         <v>8</v>
       </c>
       <c r="K58" s="62" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L58" s="29">
         <v>1E-3</v>
@@ -4719,31 +4718,31 @@
         <v>50</v>
       </c>
       <c r="C59" s="86" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="D59" s="87" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E59" s="88" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="F59" s="87" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="G59" s="88" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="H59" s="87" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="I59" s="88" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="J59" s="87">
         <v>1</v>
       </c>
       <c r="K59" s="90" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="L59" s="89">
         <v>1.8360000000000001E-2</v>
@@ -4760,31 +4759,31 @@
         <v>51</v>
       </c>
       <c r="C60" s="82" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="D60" s="83" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="E60" s="84" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="F60" s="83" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="G60" s="84" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="H60" s="83" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="I60" s="84" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="J60" s="83">
         <v>1</v>
       </c>
       <c r="K60" s="85" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L60" s="76">
         <v>1.2999999999999999E-3</v>
@@ -4801,31 +4800,31 @@
         <v>52</v>
       </c>
       <c r="C61" s="86" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="D61" s="87" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E61" s="88" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="F61" s="87" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="G61" s="88" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="H61" s="87" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="I61" s="88" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="J61" s="87">
         <v>1</v>
       </c>
       <c r="K61" s="90" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="L61" s="89">
         <v>0.22950000000000001</v>
@@ -4842,31 +4841,31 @@
         <v>53</v>
       </c>
       <c r="C62" s="82" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="D62" s="83" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="E62" s="84" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="F62" s="83" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="G62" s="84" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="H62" s="83" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="I62" s="84" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="J62" s="83">
         <v>1</v>
       </c>
       <c r="K62" s="85" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L62" s="76">
         <v>1.4E-3</v>
@@ -4883,31 +4882,31 @@
         <v>54</v>
       </c>
       <c r="C63" s="86" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="D63" s="87" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E63" s="88" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="F63" s="87" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="G63" s="88" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="H63" s="87" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="I63" s="88" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="J63" s="87">
         <v>1</v>
       </c>
       <c r="K63" s="90" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="L63" s="89">
         <v>0.1</v>
@@ -4924,31 +4923,31 @@
         <v>55</v>
       </c>
       <c r="C64" s="82" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="D64" s="83" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E64" s="84" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="F64" s="83" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="G64" s="84" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="H64" s="83" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="I64" s="84" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="J64" s="83">
         <v>1</v>
       </c>
       <c r="K64" s="85" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L64" s="76">
         <v>4.1000000000000003E-3</v>
@@ -4965,31 +4964,31 @@
         <v>56</v>
       </c>
       <c r="C65" s="86" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="D65" s="87" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E65" s="88" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="F65" s="87" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="G65" s="88" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="H65" s="87" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="I65" s="88" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="J65" s="87">
         <v>1</v>
       </c>
       <c r="K65" s="90" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L65" s="89">
         <v>1.2999999999999999E-3</v>
@@ -5006,31 +5005,31 @@
         <v>57</v>
       </c>
       <c r="C66" s="82" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="D66" s="83" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E66" s="84" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="F66" s="83" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="G66" s="83" t="s">
-        <v>334</v>
+        <v>329</v>
       </c>
       <c r="H66" s="83" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="I66" s="84" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="J66" s="83">
         <v>1</v>
       </c>
       <c r="K66" s="85" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L66" s="76">
         <v>7.3000000000000001E-3</v>
@@ -5047,31 +5046,31 @@
         <v>58</v>
       </c>
       <c r="C67" s="86" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="D67" s="87" t="s">
-        <v>375</v>
+        <v>369</v>
       </c>
       <c r="E67" s="88" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="F67" s="87" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="G67" s="88" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="H67" s="87" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="I67" s="88" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="J67" s="87">
         <v>2</v>
       </c>
       <c r="K67" s="90" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L67" s="89">
         <v>1.1000000000000001E-3</v>
@@ -5088,31 +5087,31 @@
         <v>59</v>
       </c>
       <c r="C68" s="48" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="D68" s="29" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E68" s="30" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="F68" s="29" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="G68" s="30" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="H68" s="29" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="I68" s="30" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="J68" s="29">
         <v>2</v>
       </c>
       <c r="K68" s="50" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L68" s="33">
         <v>1.2999999999999999E-3</v>
@@ -5129,31 +5128,31 @@
         <v>60</v>
       </c>
       <c r="C69" s="47" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="D69" s="69" t="s">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="E69" s="32" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="F69" s="31" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="G69" s="32" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="H69" s="31" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="I69" s="32" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="J69" s="31">
         <v>1</v>
       </c>
       <c r="K69" s="51" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L69" s="34">
         <v>1.1999999999999999E-3</v>
@@ -5170,31 +5169,31 @@
         <v>61</v>
       </c>
       <c r="C70" s="48" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="D70" s="29" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E70" s="30" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="F70" s="29" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="G70" s="30" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="H70" s="29" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="I70" s="30" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="J70" s="29">
         <v>2</v>
       </c>
       <c r="K70" s="50" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L70" s="33">
         <v>1.2999999999999999E-3</v>
@@ -5211,31 +5210,31 @@
         <v>62</v>
       </c>
       <c r="C71" s="47" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="D71" s="31" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E71" s="32" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="F71" s="31" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="G71" s="32" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="H71" s="31" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="I71" s="32" t="s">
-        <v>286</v>
+        <v>282</v>
       </c>
       <c r="J71" s="31">
         <v>1</v>
       </c>
       <c r="K71" s="51" t="s">
-        <v>335</v>
+        <v>330</v>
       </c>
       <c r="L71" s="34">
         <v>9.0200000000000002E-2</v>
@@ -5252,31 +5251,31 @@
         <v>63</v>
       </c>
       <c r="C72" s="48" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="D72" s="29" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E72" s="30" t="s">
-        <v>350</v>
+        <v>345</v>
       </c>
       <c r="F72" s="68" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="G72" s="30" t="s">
-        <v>364</v>
+        <v>358</v>
       </c>
       <c r="H72" s="29" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="I72" s="30" t="s">
-        <v>363</v>
+        <v>357</v>
       </c>
       <c r="J72" s="29">
         <v>1</v>
       </c>
       <c r="K72" s="50" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L72" s="33">
         <v>2.8E-3</v>
@@ -5293,31 +5292,31 @@
         <v>64</v>
       </c>
       <c r="C73" s="47" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="D73" s="31" t="s">
-        <v>365</v>
+        <v>359</v>
       </c>
       <c r="E73" s="32" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="F73" s="31" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="G73" s="32" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="H73" s="31" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="I73" s="32" t="s">
-        <v>290</v>
+        <v>286</v>
       </c>
       <c r="J73" s="31">
         <v>6</v>
       </c>
       <c r="K73" s="51" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L73" s="34">
         <v>1E-3</v>
@@ -5334,31 +5333,31 @@
         <v>65</v>
       </c>
       <c r="C74" s="48" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="D74" s="29" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E74" s="30" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="F74" s="29" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="G74" s="30" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="H74" s="29" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="I74" s="30" t="s">
-        <v>287</v>
+        <v>283</v>
       </c>
       <c r="J74" s="29">
         <v>1</v>
       </c>
       <c r="K74" s="50" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L74" s="33">
         <v>1E-3</v>
@@ -5375,31 +5374,31 @@
         <v>66</v>
       </c>
       <c r="C75" s="47" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="D75" s="31" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E75" s="32" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="F75" s="31" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="G75" s="32" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="H75" s="31" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="I75" s="32" t="s">
-        <v>288</v>
+        <v>284</v>
       </c>
       <c r="J75" s="31">
         <v>1</v>
       </c>
       <c r="K75" s="51" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L75" s="34">
         <v>3.8E-3</v>
@@ -5416,31 +5415,31 @@
         <v>67</v>
       </c>
       <c r="C76" s="77" t="s">
-        <v>308</v>
+        <v>304</v>
       </c>
       <c r="D76" s="78" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E76" s="79" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="F76" s="78" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="G76" s="79" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="H76" s="78" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="I76" s="79" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="J76" s="78">
         <v>4</v>
       </c>
       <c r="K76" s="80" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L76" s="52">
         <v>1E-3</v>
@@ -5449,7 +5448,7 @@
         <v>0.1</v>
       </c>
       <c r="N76" s="52" t="s">
-        <v>366</v>
+        <v>360</v>
       </c>
     </row>
     <row r="77" spans="1:14" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -5459,38 +5458,38 @@
         <v>68</v>
       </c>
       <c r="C77" s="77" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="D77" s="96" t="s">
-        <v>392</v>
+        <v>386</v>
       </c>
       <c r="E77" s="79" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="F77" s="78" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="G77" s="79" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="H77" s="78" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="I77" s="79" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="J77" s="78">
         <v>11</v>
       </c>
       <c r="K77" s="52" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="L77" s="52"/>
       <c r="M77" s="52" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="N77" s="52" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
     </row>
     <row r="78" spans="1:14" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -5500,31 +5499,31 @@
         <v>69</v>
       </c>
       <c r="C78" s="82" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
       <c r="D78" s="83" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E78" s="84" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="F78" s="83" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="G78" s="84" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="H78" s="83" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="I78" s="84" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="J78" s="83">
         <v>1</v>
       </c>
       <c r="K78" s="85" t="s">
-        <v>400</v>
+        <v>394</v>
       </c>
       <c r="L78" s="76">
         <v>1.42</v>
@@ -5542,31 +5541,31 @@
         <v>70</v>
       </c>
       <c r="C79" s="86" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="D79" s="87" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E79" s="88" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="F79" s="87" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="G79" s="88">
         <v>750314597</v>
       </c>
       <c r="H79" s="87" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="I79" s="88" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="J79" s="87">
         <v>1</v>
       </c>
       <c r="K79" s="90" t="s">
-        <v>328</v>
+        <v>324</v>
       </c>
       <c r="L79" s="89">
         <v>3.57</v>
@@ -5583,31 +5582,31 @@
         <v>71</v>
       </c>
       <c r="C80" s="82" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="D80" s="83" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E80" s="84" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="F80" s="83" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="G80" s="84" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="H80" s="83" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="I80" s="84" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="J80" s="83">
         <v>1</v>
       </c>
       <c r="K80" s="85" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L80" s="76">
         <v>2.2098</v>
@@ -5624,31 +5623,31 @@
         <v>72</v>
       </c>
       <c r="C81" s="86" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="D81" s="87" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E81" s="88" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="F81" s="87" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="G81" s="87" t="s">
-        <v>337</v>
+        <v>332</v>
       </c>
       <c r="H81" s="87" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="I81" s="88" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="J81" s="87">
         <v>1</v>
       </c>
       <c r="K81" s="90" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L81" s="89">
         <v>0.8448</v>
@@ -5665,31 +5664,31 @@
         <v>73</v>
       </c>
       <c r="C82" s="82" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="D82" s="83" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="E82" s="84" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="F82" s="83" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="G82" s="83" t="s">
-        <v>338</v>
+        <v>333</v>
       </c>
       <c r="H82" s="83" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="I82" s="84" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="J82" s="83">
         <v>1</v>
       </c>
       <c r="K82" s="85" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L82" s="76">
         <v>0.6825</v>
@@ -5706,31 +5705,31 @@
         <v>74</v>
       </c>
       <c r="C83" s="86" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="D83" s="87" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E83" s="88" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="F83" s="87" t="s">
+        <v>290</v>
+      </c>
+      <c r="G83" s="88" t="s">
+        <v>165</v>
+      </c>
+      <c r="H83" s="87" t="s">
+        <v>238</v>
+      </c>
+      <c r="I83" s="88" t="s">
         <v>294</v>
-      </c>
-      <c r="G83" s="88" t="s">
-        <v>168</v>
-      </c>
-      <c r="H83" s="87" t="s">
-        <v>241</v>
-      </c>
-      <c r="I83" s="88" t="s">
-        <v>298</v>
       </c>
       <c r="J83" s="87">
         <v>1</v>
       </c>
       <c r="K83" s="90" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L83" s="89">
         <v>0.89890000000000003</v>
@@ -5747,31 +5746,31 @@
         <v>75</v>
       </c>
       <c r="C84" s="82" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="D84" s="83" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="E84" s="84" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="F84" s="83" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="G84" s="84" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="H84" s="83" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="I84" s="84" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="J84" s="83">
         <v>1</v>
       </c>
       <c r="K84" s="85" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L84" s="76">
         <v>0.39779999999999999</v>
@@ -5788,31 +5787,31 @@
         <v>76</v>
       </c>
       <c r="C85" s="53" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="D85" s="54" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E85" s="55" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="F85" s="54" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="G85" s="55" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="H85" s="54" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="I85" s="55" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="J85" s="54">
         <v>1</v>
       </c>
       <c r="K85" s="57" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L85" s="56">
         <v>5.5602999999999998</v>
@@ -5821,7 +5820,7 @@
         <v>5.5602999999999998</v>
       </c>
       <c r="N85" s="56" t="s">
-        <v>352</v>
+        <v>347</v>
       </c>
     </row>
     <row r="86" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -5831,31 +5830,31 @@
         <v>77</v>
       </c>
       <c r="C86" s="82" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="D86" s="83" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E86" s="84" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="F86" s="83" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="G86" s="84" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="H86" s="83" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="I86" s="93" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="J86" s="83">
         <v>1</v>
       </c>
       <c r="K86" s="85" t="s">
-        <v>336</v>
+        <v>331</v>
       </c>
       <c r="L86" s="76">
         <v>2.6459999999999999</v>
@@ -5872,31 +5871,31 @@
         <v>78</v>
       </c>
       <c r="C87" s="86" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="D87" s="87" t="s">
-        <v>367</v>
+        <v>361</v>
       </c>
       <c r="E87" s="88" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="F87" s="87" t="s">
-        <v>295</v>
+        <v>291</v>
       </c>
       <c r="G87" s="87" t="s">
-        <v>339</v>
+        <v>334</v>
       </c>
       <c r="H87" s="87" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="I87" s="88" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="J87" s="94">
         <v>2</v>
       </c>
       <c r="K87" s="90" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L87" s="89">
         <v>1.8487</v>
@@ -5913,31 +5912,31 @@
         <v>79</v>
       </c>
       <c r="C88" s="48" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="D88" s="29" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E88" s="30" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="F88" s="29" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="G88" s="30" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="H88" s="29" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="I88" s="30" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="J88" s="29">
         <v>1</v>
       </c>
       <c r="K88" s="50" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L88" s="33">
         <v>0.45979999999999999</v>
@@ -5954,31 +5953,31 @@
         <v>80</v>
       </c>
       <c r="C89" s="47" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="D89" s="31" t="s">
-        <v>368</v>
+        <v>362</v>
       </c>
       <c r="E89" s="32" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="F89" s="31" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="G89" s="31" t="s">
-        <v>340</v>
+        <v>335</v>
       </c>
       <c r="H89" s="31" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="I89" s="32" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="J89" s="31">
         <v>1</v>
       </c>
       <c r="K89" s="51" t="s">
-        <v>341</v>
+        <v>336</v>
       </c>
       <c r="L89" s="34">
         <v>3.93</v>
@@ -5995,29 +5994,29 @@
         <v>81</v>
       </c>
       <c r="C90" s="47" t="s">
-        <v>383</v>
+        <v>377</v>
       </c>
       <c r="D90" s="31" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="E90" s="32" t="s">
-        <v>386</v>
+        <v>380</v>
       </c>
       <c r="F90" s="31" t="s">
-        <v>292</v>
+        <v>288</v>
       </c>
       <c r="G90" s="32" t="s">
-        <v>384</v>
+        <v>378</v>
       </c>
       <c r="H90" s="31" t="s">
-        <v>385</v>
+        <v>379</v>
       </c>
       <c r="I90" s="32"/>
       <c r="J90" s="31">
         <v>1</v>
       </c>
       <c r="K90" s="51" t="s">
-        <v>319</v>
+        <v>315</v>
       </c>
       <c r="L90" s="34">
         <v>7.1199999999999999E-2</v>
@@ -6039,7 +6038,7 @@
       <c r="I91" s="102"/>
       <c r="J91" s="102"/>
       <c r="K91" s="103" t="s">
-        <v>398</v>
+        <v>392</v>
       </c>
       <c r="L91" s="104"/>
       <c r="M91" s="104">
@@ -6054,84 +6053,84 @@
     <mergeCell ref="N3:N8"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="K11" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="K12" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="K13" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="K14" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="K15" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="K16" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="K17" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="K18" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="K19" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="K21" r:id="rId10" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="K22" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="K23" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="K24" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
-    <hyperlink ref="K25" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="K26" r:id="rId15" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="K27" r:id="rId16" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="K28" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="K29" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
-    <hyperlink ref="K30" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
-    <hyperlink ref="K31" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
-    <hyperlink ref="K32" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
-    <hyperlink ref="K33" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
-    <hyperlink ref="K34" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
-    <hyperlink ref="K36" r:id="rId24" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
-    <hyperlink ref="K37" r:id="rId25" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
-    <hyperlink ref="K38" r:id="rId26" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
-    <hyperlink ref="K39" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
-    <hyperlink ref="K40" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
-    <hyperlink ref="K41" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
-    <hyperlink ref="K43" r:id="rId30" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
-    <hyperlink ref="K44" r:id="rId31" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
-    <hyperlink ref="K46" r:id="rId32" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
-    <hyperlink ref="K48" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
-    <hyperlink ref="K51" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
-    <hyperlink ref="K52" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
-    <hyperlink ref="K53" r:id="rId36" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
-    <hyperlink ref="K54" r:id="rId37" xr:uid="{00000000-0004-0000-0000-000029000000}"/>
-    <hyperlink ref="K55" r:id="rId38" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
-    <hyperlink ref="K56" r:id="rId39" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
-    <hyperlink ref="K57" r:id="rId40" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
-    <hyperlink ref="K69" r:id="rId41" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
-    <hyperlink ref="K59" r:id="rId42" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
-    <hyperlink ref="K60" r:id="rId43" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
-    <hyperlink ref="K61" r:id="rId44" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
-    <hyperlink ref="K62" r:id="rId45" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
-    <hyperlink ref="K64" r:id="rId46" xr:uid="{00000000-0004-0000-0000-000033000000}"/>
-    <hyperlink ref="K65" r:id="rId47" xr:uid="{00000000-0004-0000-0000-000034000000}"/>
-    <hyperlink ref="K66" r:id="rId48" xr:uid="{00000000-0004-0000-0000-000035000000}"/>
-    <hyperlink ref="K67" r:id="rId49" xr:uid="{00000000-0004-0000-0000-000036000000}"/>
-    <hyperlink ref="K68" r:id="rId50" xr:uid="{00000000-0004-0000-0000-000037000000}"/>
-    <hyperlink ref="K70" r:id="rId51" xr:uid="{00000000-0004-0000-0000-000038000000}"/>
-    <hyperlink ref="K71" r:id="rId52" xr:uid="{00000000-0004-0000-0000-000039000000}"/>
-    <hyperlink ref="K72" r:id="rId53" xr:uid="{00000000-0004-0000-0000-00003A000000}"/>
-    <hyperlink ref="K75" r:id="rId54" xr:uid="{00000000-0004-0000-0000-00003B000000}"/>
-    <hyperlink ref="K76" r:id="rId55" xr:uid="{00000000-0004-0000-0000-00003C000000}"/>
-    <hyperlink ref="K73" r:id="rId56" xr:uid="{00000000-0004-0000-0000-00003D000000}"/>
-    <hyperlink ref="K79" r:id="rId57" xr:uid="{00000000-0004-0000-0000-00003E000000}"/>
-    <hyperlink ref="K81" r:id="rId58" xr:uid="{00000000-0004-0000-0000-000040000000}"/>
-    <hyperlink ref="K82" r:id="rId59" xr:uid="{00000000-0004-0000-0000-000041000000}"/>
-    <hyperlink ref="K84" r:id="rId60" xr:uid="{00000000-0004-0000-0000-000043000000}"/>
-    <hyperlink ref="K85" r:id="rId61" xr:uid="{00000000-0004-0000-0000-000044000000}"/>
-    <hyperlink ref="K86" r:id="rId62" xr:uid="{00000000-0004-0000-0000-000045000000}"/>
-    <hyperlink ref="K87" r:id="rId63" xr:uid="{00000000-0004-0000-0000-000046000000}"/>
-    <hyperlink ref="K89" r:id="rId64" xr:uid="{00000000-0004-0000-0000-000047000000}"/>
-    <hyperlink ref="K88" r:id="rId65" xr:uid="{00000000-0004-0000-0000-000048000000}"/>
-    <hyperlink ref="K58" r:id="rId66" xr:uid="{00000000-0004-0000-0000-000049000000}"/>
-    <hyperlink ref="K47" r:id="rId67" xr:uid="{00000000-0004-0000-0000-00004A000000}"/>
-    <hyperlink ref="K90" r:id="rId68" xr:uid="{00000000-0004-0000-0000-00004B000000}"/>
-    <hyperlink ref="K42" r:id="rId69" xr:uid="{00000000-0004-0000-0000-00004C000000}"/>
-    <hyperlink ref="K10" r:id="rId70" xr:uid="{A8906534-0257-42E0-9364-25FFD226DFF8}"/>
-    <hyperlink ref="K20" r:id="rId71" xr:uid="{FEBC96A2-AC9F-4433-8C7D-5304408C186D}"/>
-    <hyperlink ref="K35" r:id="rId72" xr:uid="{D6467D42-343A-42A6-B59B-5940B00CEAEE}"/>
-    <hyperlink ref="K45" r:id="rId73" xr:uid="{4843D163-9805-4AF6-AB48-0FB2B0C8B803}"/>
-    <hyperlink ref="K63" r:id="rId74" xr:uid="{CFF4AE3A-6BDB-4D47-B838-8749D726282A}"/>
-    <hyperlink ref="K80" r:id="rId75" xr:uid="{3134D4B0-2206-4CB1-9A6A-3F755F123261}"/>
-    <hyperlink ref="K83" r:id="rId76" xr:uid="{97B0841F-B518-4D3B-92E8-7CFF723AF904}"/>
-    <hyperlink ref="K50" r:id="rId77" xr:uid="{2535B222-222C-4C4F-BBA3-B1169AA89BB2}"/>
-    <hyperlink ref="K78" r:id="rId78" xr:uid="{3476FBDB-7D07-4094-8729-F4DB1B92AF43}"/>
+    <hyperlink ref="K11" r:id="rId1"/>
+    <hyperlink ref="K12" r:id="rId2"/>
+    <hyperlink ref="K13" r:id="rId3"/>
+    <hyperlink ref="K14" r:id="rId4"/>
+    <hyperlink ref="K15" r:id="rId5"/>
+    <hyperlink ref="K16" r:id="rId6"/>
+    <hyperlink ref="K17" r:id="rId7"/>
+    <hyperlink ref="K18" r:id="rId8"/>
+    <hyperlink ref="K19" r:id="rId9"/>
+    <hyperlink ref="K21" r:id="rId10"/>
+    <hyperlink ref="K22" r:id="rId11"/>
+    <hyperlink ref="K23" r:id="rId12"/>
+    <hyperlink ref="K24" r:id="rId13"/>
+    <hyperlink ref="K25" r:id="rId14"/>
+    <hyperlink ref="K26" r:id="rId15"/>
+    <hyperlink ref="K27" r:id="rId16"/>
+    <hyperlink ref="K28" r:id="rId17"/>
+    <hyperlink ref="K29" r:id="rId18"/>
+    <hyperlink ref="K30" r:id="rId19"/>
+    <hyperlink ref="K31" r:id="rId20"/>
+    <hyperlink ref="K32" r:id="rId21"/>
+    <hyperlink ref="K33" r:id="rId22"/>
+    <hyperlink ref="K34" r:id="rId23"/>
+    <hyperlink ref="K36" r:id="rId24"/>
+    <hyperlink ref="K37" r:id="rId25"/>
+    <hyperlink ref="K38" r:id="rId26"/>
+    <hyperlink ref="K39" r:id="rId27"/>
+    <hyperlink ref="K40" r:id="rId28"/>
+    <hyperlink ref="K41" r:id="rId29"/>
+    <hyperlink ref="K43" r:id="rId30"/>
+    <hyperlink ref="K44" r:id="rId31"/>
+    <hyperlink ref="K46" r:id="rId32"/>
+    <hyperlink ref="K48" r:id="rId33"/>
+    <hyperlink ref="K51" r:id="rId34"/>
+    <hyperlink ref="K52" r:id="rId35"/>
+    <hyperlink ref="K53" r:id="rId36"/>
+    <hyperlink ref="K54" r:id="rId37"/>
+    <hyperlink ref="K55" r:id="rId38"/>
+    <hyperlink ref="K56" r:id="rId39"/>
+    <hyperlink ref="K69" r:id="rId40"/>
+    <hyperlink ref="K59" r:id="rId41"/>
+    <hyperlink ref="K60" r:id="rId42"/>
+    <hyperlink ref="K61" r:id="rId43"/>
+    <hyperlink ref="K62" r:id="rId44"/>
+    <hyperlink ref="K64" r:id="rId45"/>
+    <hyperlink ref="K65" r:id="rId46"/>
+    <hyperlink ref="K66" r:id="rId47"/>
+    <hyperlink ref="K67" r:id="rId48"/>
+    <hyperlink ref="K68" r:id="rId49"/>
+    <hyperlink ref="K70" r:id="rId50"/>
+    <hyperlink ref="K71" r:id="rId51"/>
+    <hyperlink ref="K72" r:id="rId52"/>
+    <hyperlink ref="K75" r:id="rId53"/>
+    <hyperlink ref="K76" r:id="rId54"/>
+    <hyperlink ref="K73" r:id="rId55"/>
+    <hyperlink ref="K79" r:id="rId56"/>
+    <hyperlink ref="K81" r:id="rId57"/>
+    <hyperlink ref="K82" r:id="rId58"/>
+    <hyperlink ref="K84" r:id="rId59"/>
+    <hyperlink ref="K85" r:id="rId60"/>
+    <hyperlink ref="K86" r:id="rId61"/>
+    <hyperlink ref="K87" r:id="rId62"/>
+    <hyperlink ref="K89" r:id="rId63"/>
+    <hyperlink ref="K88" r:id="rId64"/>
+    <hyperlink ref="K58" r:id="rId65"/>
+    <hyperlink ref="K47" r:id="rId66"/>
+    <hyperlink ref="K90" r:id="rId67"/>
+    <hyperlink ref="K42" r:id="rId68"/>
+    <hyperlink ref="K10" r:id="rId69"/>
+    <hyperlink ref="K20" r:id="rId70"/>
+    <hyperlink ref="K35" r:id="rId71"/>
+    <hyperlink ref="K45" r:id="rId72"/>
+    <hyperlink ref="K63" r:id="rId73"/>
+    <hyperlink ref="K80" r:id="rId74"/>
+    <hyperlink ref="K83" r:id="rId75"/>
+    <hyperlink ref="K50" r:id="rId76"/>
+    <hyperlink ref="K78" r:id="rId77"/>
+    <hyperlink ref="K57" r:id="rId78"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId79"/>

</xml_diff>